<commit_message>
Refine split OPP column script and updated Excel output
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAY6zK7UD2j9ggDmqRx5EG
</commit_message>
<xml_diff>
--- a/OPP_Quality_Analysis_Updated.xlsx
+++ b/OPP_Quality_Analysis_Updated.xlsx
@@ -849,10 +849,14 @@
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Prerequisites section — 'Access to Both Phones' prerequisite conflicts with the most common real-world scenario.
-The vast majority of tickets (INC0036041, INC0017694, INC0017809, INC0015306, INC0024035, INC0016202) involve users who have already switched to a new phone and no longer have the old one. The prerequisite states 'Ensure you have both your old phone,' yet the very next sub-section says to raise an incident if you don't. Restructure the document with two clearly-labelled paths at the top: Path A — Old phone still available (self-service) and Path B — Old phone not available (service desk-assisted reset).</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr"/>
+The vast majority of tickets (INC0036041, INC0017694, INC0017809, INC0015306, INC0024035, INC0016202) involve users who have already switched to a new phone and no longer have the old one. The prerequisite states 'Ensure you have both your old phone,' yet the very next sub-section says to raise an incident if you don't.</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Restructure the document with two clearly-labelled paths at the top: Path A — Old phone still available (self-service) and Path B — Old phone not available (service desk-assisted reset).</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -1124,10 +1128,14 @@
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Approval Steps, Step 13 — No guidance on what to do when automated provisioning fails after approval.
-Tickets INC0093752, INC0091492, INC0167458, INC0167459 (all 'Request Closure API failed') show that even after a role owner approves, backend provisioning can fail, leaving users without access. The OPP ends at 'changes to the role will become active.' Add a post-approval monitoring note: how to confirm provisioning succeeded (via Request History), what a provisioning failure looks like, and that an incident should be raised if tasks remain in a failed state beyond SLA.</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr"/>
+Tickets INC0093752, INC0091492, INC0167458, INC0167459 (all 'Request Closure API failed') show that even after a role owner approves, backend provisioning can fail, leaving users without access. The OPP ends at 'changes to the role will become active.'</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Add a post-approval monitoring note: how to confirm provisioning succeeded (via Request History), what a provisioning failure looks like, and that an incident should be raised if tasks remain in a failed state beyond SLA.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="120" customHeight="1">
       <c r="A19" s="9" t="n">
@@ -1182,10 +1190,14 @@
       <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Role Creation Step 11 vs Role-Service Profile Mapping Update Step 10 — Entitlement type list is inconsistent between sections.
-The Role Creation section lists SportsEntriesAndQualifications_PreProd but omits RiskIQ: Group, which appears in the Mapping Update section. This inconsistency can cause role owners to miss valid entitlement options. Align both lists and maintain a single master entitlement type table that both sections reference, so it needs only one update point as new systems are onboarded.</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr"/>
+The Role Creation section lists SportsEntriesAndQualifications_PreProd but omits RiskIQ: Group, which appears in the Mapping Update section. This inconsistency can cause role owners to miss valid entitlement options.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Align both lists and maintain a single master entitlement type table that both sections reference, so it needs only one update point as new systems are onboarded.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="10" t="n">
@@ -1302,10 +1314,14 @@
       <c r="E24" s="10" t="inlineStr">
         <is>
           <t>FAQ Q1 — Training completion dependency for D.TEC users creates invisible hold that requestors cannot monitor.
-INC0015119 ('onboarding shows complete but users do not yet have access 7+ days after the request') and INC0034447 ('newly onboarded SNOW users can only see Logout successful screen') show requestors are unaware of the mandatory training gate. The FAQ mentions training in passing but gives no SLA, no way to check training status, and no escalation path. Expand Q1 or add a new FAQ: 'How do I know if the mandatory training has been triggered and completed?' with steps to check training status and the expected provisioning timeline after completion.</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr"/>
+INC0015119 ('onboarding shows complete but users do not yet have access 7+ days after the request') and INC0034447 ('newly onboarded SNOW users can only see Logout successful screen') show requestors are unaware of the mandatory training gate. The FAQ mentions training in passing but gives no SLA, no way to check training status, and no escalation path.</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Expand Q1 or add a new FAQ: 'How do I know if the mandatory training has been triggered and completed?' with steps to check training status and the expected provisioning timeline after completion.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="120" customHeight="1">
       <c r="A25" s="10" t="n">
@@ -1329,10 +1345,14 @@
       <c r="E25" s="10" t="inlineStr">
         <is>
           <t>FAQ Q3 — Role Update approver logic is described, but the 'Invalid role' failure path is absent.
-INC0026826 and INC0042868 (both errorCode:1 — 'Invalid role found in request') and INC0054691 ('username not present') show that role update requests fail silently when the role name is invalid or the user account is in the wrong state. FAQ Q3 ends at 'Once approved, the roles will automatically be assigned.' Add a note: 'If a role update request fails, an incident will be raised automatically. Common causes: the role name is inactive in Saviynt, the user account is inactive, or a duplicate active account exists. Check the RITM for error details or raise an incident with the IAM team.'</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr"/>
+INC0026826 and INC0042868 (both errorCode:1 — 'Invalid role found in request') and INC0054691 ('username not present') show that role update requests fail silently when the role name is invalid or the user account is in the wrong state. FAQ Q3 ends at 'Once approved, the roles will automatically be assigned.'</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Add a note: 'If a role update request fails, an incident will be raised automatically. Common causes: the role name is inactive in Saviynt, the user account is inactive, or a duplicate active account exists. Check the RITM for error details or raise an incident with the IAM team.'</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="120" customHeight="1">
       <c r="A26" s="10" t="n">

</xml_diff>